<commit_message>
Added Test Cases for Multibill Registration and Email Text to Pay
</commit_message>
<xml_diff>
--- a/KatalonData/BWPBootstrapData/BWPCCData.xlsx
+++ b/KatalonData/BWPBootstrapData/BWPCCData.xlsx
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="87">
   <si>
     <t>Result</t>
   </si>
@@ -298,6 +298,21 @@
   </si>
   <si>
     <t>Fri Nov 21 00:30:17 IST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 20:37:01 EST 2025</t>
+  </si>
+  <si>
+    <t>Wed Dec 10 20:38:06 EST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 12:24:14 EST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 12:31:52 EST 2025</t>
+  </si>
+  <si>
+    <t>Mon Dec 15 14:42:01 EST 2025</t>
   </si>
 </sst>
 </file>
@@ -687,7 +702,7 @@
         <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">
@@ -2164,7 +2179,7 @@
         <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="1" t="s">

</xml_diff>